<commit_message>
Fix final evaluation reuse and complete reproducible submission evidence
</commit_message>
<xml_diff>
--- a/submissions/2A202602395_DoanQuangThang/results.xlsx
+++ b/submissions/2A202602395_DoanQuangThang/results.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Backbones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Final" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PerClass" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Latency" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$R$6</definedName>
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$T$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$J$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -89,6 +89,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2866,12 +2869,6 @@
       <c r="N2" s="2" t="n">
         <v>0.08661136645899828</v>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2926,12 +2923,6 @@
       <c r="N3" s="2" t="n">
         <v>0.0114093903316874</v>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2986,12 +2977,6 @@
       <c r="N4" s="2" t="n">
         <v>0.08661136645899828</v>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3046,12 +3031,6 @@
       <c r="N5" s="2" t="n">
         <v>0.08540676027295392</v>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3106,12 +3085,6 @@
       <c r="N6" s="2" t="n">
         <v>0.01495680634639824</v>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3166,12 +3139,6 @@
       <c r="N7" s="2" t="n">
         <v>0.08540676027295392</v>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3286,12 +3253,6 @@
       <c r="N9" s="2" t="n">
         <v>0.01201481085183027</v>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3346,12 +3307,6 @@
       <c r="N10" s="2" t="n">
         <v>0.08699897879925093</v>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3364,12 +3319,6 @@
           <t>mean ± sample std</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" s="2" t="n">
         <v>0.9710163391463134</v>
       </c>
@@ -3385,7 +3334,6 @@
       <c r="M11" s="2" t="n">
         <v>0.00582055958839401</v>
       </c>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" s="2" t="n">
         <v>3</v>
       </c>
@@ -3416,12 +3364,6 @@
           <t>mean ± sample std</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" s="2" t="n">
         <v>0.9681781122353955</v>
       </c>
@@ -3437,7 +3379,6 @@
       <c r="M12" s="2" t="n">
         <v>0.01279366917663864</v>
       </c>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" s="2" t="n">
         <v>3</v>
       </c>
@@ -3468,12 +3409,6 @@
           <t>mean ± sample std</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" s="2" t="n">
         <v>0.9710163391463134</v>
       </c>
@@ -3489,7 +3424,6 @@
       <c r="M13" s="2" t="n">
         <v>0.00582055958839401</v>
       </c>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" s="2" t="n">
         <v>3</v>
       </c>
@@ -5287,7 +5221,6 @@
           <t>I00</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" s="2" t="n">
         <v>5.728163000014774</v>
       </c>
@@ -5297,9 +5230,6 @@
       <c r="E11" s="2" t="n">
         <v>10.71189014997798</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5327,8 +5257,6 @@
       <c r="O11" t="b">
         <v>0</v>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="b">
         <v>0</v>
       </c>
@@ -5339,7 +5267,6 @@
           <t>I00</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" s="2" t="n">
         <v>115.7681530000332</v>
       </c>
@@ -5403,7 +5330,6 @@
           <t>I01</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" s="2" t="n">
         <v>10.86121899999171</v>
       </c>
@@ -5413,9 +5339,6 @@
       <c r="E13" s="2" t="n">
         <v>12.06298938996838</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5443,8 +5366,6 @@
       <c r="O13" t="b">
         <v>0</v>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="b">
         <v>0</v>
       </c>
@@ -5455,7 +5376,6 @@
           <t>I01</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" s="2" t="n">
         <v>249.52232250007</v>
       </c>
@@ -5519,7 +5439,6 @@
           <t>I02</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="2" t="n">
         <v>11.17918400001372</v>
       </c>
@@ -5529,9 +5448,6 @@
       <c r="E15" s="2" t="n">
         <v>12.03826149994029</v>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5559,8 +5475,6 @@
       <c r="O15" t="b">
         <v>0</v>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="b">
         <v>0</v>
       </c>
@@ -5571,7 +5485,6 @@
           <t>I02</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="2" t="n">
         <v>275.8866594999745</v>
       </c>
@@ -5635,7 +5548,6 @@
           <t>I03</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="2" t="n">
         <v>27.80482650001659</v>
       </c>
@@ -5645,9 +5557,6 @@
       <c r="E17" s="2" t="n">
         <v>30.18748068996842</v>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5675,8 +5584,6 @@
       <c r="O17" t="b">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="b">
         <v>0</v>
       </c>
@@ -5687,7 +5594,6 @@
           <t>I03</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="2" t="n">
         <v>679.7784954999884</v>
       </c>
@@ -5751,7 +5657,6 @@
           <t>I04</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" s="2" t="n">
         <v>6.6624335000256</v>
       </c>
@@ -5761,9 +5666,6 @@
       <c r="E19" s="2" t="n">
         <v>9.562904129981003</v>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5791,8 +5693,6 @@
       <c r="O19" t="b">
         <v>0</v>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="b">
         <v>0</v>
       </c>
@@ -5803,7 +5703,6 @@
           <t>I04</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" s="2" t="n">
         <v>173.188314000015</v>
       </c>
@@ -5867,7 +5766,6 @@
           <t>I05</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" s="2" t="n">
         <v>6.03289550002728</v>
       </c>
@@ -5877,9 +5775,6 @@
       <c r="E21" s="2" t="n">
         <v>7.0171876800282</v>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -5907,8 +5802,6 @@
       <c r="O21" t="b">
         <v>0</v>
       </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="b">
         <v>0</v>
       </c>
@@ -5919,7 +5812,6 @@
           <t>I05</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" s="2" t="n">
         <v>137.0123770000191</v>
       </c>
@@ -5983,7 +5875,6 @@
           <t>I06</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" s="2" t="n">
         <v>8.096603500007404</v>
       </c>
@@ -5993,9 +5884,6 @@
       <c r="E23" s="2" t="n">
         <v>8.809600529995123</v>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>Tesla T4</t>
@@ -6023,8 +5911,6 @@
       <c r="O23" t="b">
         <v>0</v>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="b">
         <v>0</v>
       </c>
@@ -6035,7 +5921,6 @@
           <t>I06</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" s="2" t="n">
         <v>49.05601650000335</v>
       </c>
@@ -6105,15 +5990,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6147,6 +6038,36 @@
           <t>latency_ms</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>latency_percentile</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>latency_source</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>params_m</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>gmac</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>train_seconds_per_epoch</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>is_baseline</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6173,6 +6094,28 @@
       <c r="F2" s="2" t="n">
         <v>28.74660980005501</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>I03: batch 1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6199,6 +6142,28 @@
       <c r="F3" s="2" t="n">
         <v>8.641239550064483</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>I04: batch 1</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6225,6 +6190,28 @@
       <c r="F4" s="2" t="n">
         <v>11.82462514997269</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>I02: batch 1</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6251,6 +6238,28 @@
       <c r="F5" s="2" t="n">
         <v>11.60492939995947</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>I01: batch 1</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6277,30 +6286,76 @@
       <c r="F6" s="2" t="n">
         <v>8.639485649973722</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>I06: batch 1</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>T05</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>training</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>convnext_tiny</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="4" t="n">
         <v>0.9721130318872303</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="4" t="n">
         <v>0.9785775492716366</v>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" s="4" t="n">
+        <v>5.728163000014774</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>I00: đúng checkpoint seed đầu, single-view</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>4.469676288</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>66.23328104330002</v>
+      </c>
+      <c r="L7" s="3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6327,6 +6382,28 @@
       <c r="F8" s="2" t="n">
         <v>9.41591475000223</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>I00: batch 1</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6353,6 +6430,28 @@
       <c r="F9" s="2" t="n">
         <v>6.483059749973562</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>I05: batch 1</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6376,7 +6475,33 @@
       <c r="E10" s="2" t="n">
         <v>0.9782919165952585</v>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Chưa đo riêng</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Chưa đo</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Chưa đo riêng</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>4.469676288</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>66.46373123600024</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6400,8 +6525,89 @@
       <c r="E11" s="2" t="n">
         <v>0.9782919165952585</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-    </row>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Chưa đo riêng</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Chưa đo</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Chưa đo riêng</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>4.469676288</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>66.44768587019989</v>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>training</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.9693657717968429</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.9765781205369894</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>5.751443500003006</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>T00: single-view, seed đầu vòng cuối</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>4.469676288</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>65.75213859979995</v>
+      </c>
+      <c r="L12" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
@@ -6411,7 +6617,7 @@
       <c r="F20" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:L20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>